<commit_message>
Till 21st Jan 25
</commit_message>
<xml_diff>
--- a/TestData/T2362_TMTC0003198_VerifyModificationOfLOBValueForGivenOpportunity.xlsx
+++ b/TestData/T2362_TMTC0003198_VerifyModificationOfLOBValueForGivenOpportunity.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28129"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\SGoyal0427\source\repos\SF_Automation\TestData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B687F8F1-BC77-40A6-85D9-24267C028AA8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9CC8D846-1637-4EAB-9CFF-C289AB7D2C48}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView showHorizontalScroll="0" showVerticalScroll="0" xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView showHorizontalScroll="0" showVerticalScroll="0" xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="AddOpportunity" sheetId="1" r:id="rId1"/>
@@ -51,9 +51,6 @@
     <t>AdditonalSubject</t>
   </si>
   <si>
-    <t>BUS - Business Services</t>
-  </si>
-  <si>
     <t>No</t>
   </si>
   <si>
@@ -270,10 +267,13 @@
     <t>100000.0</t>
   </si>
   <si>
-    <t>CSDN-0000001546</t>
-  </si>
-  <si>
     <t>Karan Chopra</t>
+  </si>
+  <si>
+    <t>Dental</t>
+  </si>
+  <si>
+    <t>HC - Healthcare</t>
   </si>
 </sst>
 </file>
@@ -1091,159 +1091,159 @@
         <v>6</v>
       </c>
       <c r="H1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="I1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="I1" s="1" t="s">
-        <v>10</v>
-      </c>
       <c r="J1" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="K1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="K1" s="1" t="s">
-        <v>13</v>
-      </c>
       <c r="L1" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="M1" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="M1" s="1" t="s">
-        <v>16</v>
-      </c>
       <c r="N1" s="1" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="O1" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="P1" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="P1" s="2" t="s">
+      <c r="Q1" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="Q1" s="2" t="s">
+      <c r="R1" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="R1" s="1" t="s">
+      <c r="S1" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="S1" s="1" t="s">
-        <v>25</v>
-      </c>
       <c r="T1" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="U1" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="U1" s="1" t="s">
-        <v>28</v>
-      </c>
       <c r="V1" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="W1" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="W1" s="1" t="s">
-        <v>31</v>
-      </c>
       <c r="X1" s="1" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="Y1" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="Z1" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="Z1" s="1" t="s">
-        <v>42</v>
-      </c>
       <c r="AA1" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="AB1" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="AB1" s="1" t="s">
-        <v>47</v>
-      </c>
       <c r="AD1" s="1" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
     </row>
     <row r="2" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="B2" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="C2" s="6" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="D2" t="s">
-        <v>7</v>
+        <v>81</v>
       </c>
       <c r="E2" s="10" t="s">
         <v>80</v>
       </c>
       <c r="F2" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="G2" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="H2" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="I2" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="J2" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="K2" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="L2" t="s">
+        <v>71</v>
+      </c>
+      <c r="M2" t="s">
+        <v>16</v>
+      </c>
+      <c r="N2" t="s">
+        <v>79</v>
+      </c>
+      <c r="O2" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="P2" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="Q2" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="R2" t="s">
+        <v>25</v>
+      </c>
+      <c r="S2" t="s">
+        <v>25</v>
+      </c>
+      <c r="T2" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="U2" t="s">
+        <v>28</v>
+      </c>
+      <c r="V2" t="s">
         <v>72</v>
       </c>
-      <c r="M2" t="s">
-        <v>17</v>
-      </c>
-      <c r="N2" t="s">
-        <v>81</v>
-      </c>
-      <c r="O2" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="P2" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="Q2" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="R2" t="s">
-        <v>26</v>
-      </c>
-      <c r="S2" t="s">
-        <v>26</v>
-      </c>
-      <c r="T2" s="3" t="s">
-        <v>38</v>
-      </c>
-      <c r="U2" t="s">
-        <v>29</v>
-      </c>
-      <c r="V2" t="s">
+      <c r="W2" t="s">
+        <v>31</v>
+      </c>
+      <c r="X2" t="s">
+        <v>33</v>
+      </c>
+      <c r="Y2" t="s">
         <v>73</v>
       </c>
-      <c r="W2" t="s">
-        <v>32</v>
-      </c>
-      <c r="X2" t="s">
-        <v>34</v>
-      </c>
-      <c r="Y2" t="s">
-        <v>74</v>
-      </c>
       <c r="Z2" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="AA2" s="3" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="AB2" s="3" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="AD2" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
     </row>
   </sheetData>
@@ -1263,18 +1263,18 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>19</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>20</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="B2" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
     </row>
   </sheetData>
@@ -1297,54 +1297,54 @@
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="B1" s="1" t="s">
-        <v>36</v>
-      </c>
       <c r="C1" s="1" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D1" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="G1" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="E1" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>48</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>51</v>
-      </c>
       <c r="H1" s="1" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B2" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C2" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="D2" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="E2" t="s">
         <v>0</v>
       </c>
       <c r="F2" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="G2" t="s">
         <v>0</v>
       </c>
       <c r="H2" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
     </row>
   </sheetData>
@@ -1366,80 +1366,80 @@
   <sheetData>
     <row r="1" spans="1:4" s="1" customFormat="1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="C1" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="D1" s="1" t="s">
         <v>57</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>58</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2" s="5" t="s">
+        <v>58</v>
+      </c>
+      <c r="B2" s="5" t="s">
         <v>59</v>
       </c>
-      <c r="B2" s="5" t="s">
+      <c r="C2" t="s">
+        <v>71</v>
+      </c>
+      <c r="D2" s="6" t="s">
         <v>60</v>
-      </c>
-      <c r="C2" t="s">
-        <v>72</v>
-      </c>
-      <c r="D2" s="6" t="s">
-        <v>61</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.3">
       <c r="D3" s="7" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.3">
       <c r="D4" s="7" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.3">
       <c r="D5" s="8" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.3">
       <c r="D6" s="7" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.3">
       <c r="D7" s="7" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.3">
       <c r="D8" s="7" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.3">
       <c r="D9" s="7" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.3">
       <c r="D10" s="8" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.3">
       <c r="D11" s="7" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
     </row>
     <row r="12" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="D12" s="9" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
   </sheetData>

</xml_diff>